<commit_message>
Add AC-18 Not Applicable control to demo (scope exclusion)
The demo had no genuinely Not-Applicable control. Add AC-18 (Wireless Access)
as a documented scope exclusion — the Example System boundary has no wireless,
so AC-18 is Not Applicable (distinct from SC-7's inherited-Compliant). Demo now
shows the full status spread: Compliant, inherited-Compliant, Not Applicable,
and an unassessed multi-tenant-divergent control (AC-17). 9 controls total.
</commit_message>
<xml_diff>
--- a/demo/workbooks/DEMO_NIST_800-53r5_Example System.xlsx
+++ b/demo/workbooks/DEMO_NIST_800-53r5_Example System.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1390,13 +1390,104 @@
       </c>
       <c r="U14" s="5" t="inlineStr"/>
     </row>
+    <row r="15" ht="110" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>AC-18</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Wireless Access</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>The Example System Demo authorization boundary contains no wireless networking. All connectivity is wired within the data center enclave; wireless is not deployed and is prohibited by the system configuration baseline.</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>AC-18</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>CCI-001438</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>The organization establishes configuration requirements and authorizes wireless access to the information system.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>If wireless is present, provide the wireless configuration; otherwise document the scope exclusion.</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Confirm the boundary has no wireless components. Verify the scope-exclusion statement in the SSP.</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr"/>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Noah Jaskolski</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Not Applicable — the Example System Demo boundary deploys no wireless networking; all access is wired within the data-center enclave. Wireless is prohibited by the configuration baseline, so AC-18 does not apply to this system.</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>NIST SP 800-53 Rev. 5</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>System-Specific</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>T. Prior</t>
+        </is>
+      </c>
+      <c r="U15" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A5:U5"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="N7:N14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid status" error="Status must be Compliant, Non-Compliant, or Not Applicable." type="list">
+    <dataValidation sqref="N7:N15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid status" error="Status must be Compliant, Non-Compliant, or Not Applicable." type="list">
       <formula1>"Compliant,Non-Compliant,Not Applicable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>